<commit_message>
data: 自动同步石墨文档 2026-07-17 22:22
</commit_message>
<xml_diff>
--- a/海外客诉台账_标准化数据.xlsx
+++ b/海外客诉台账_标准化数据.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="客诉明细" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="数据字典" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客诉明细" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据字典" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
data: 自动同步石墨文档 2026-07-17 16:55
</commit_message>
<xml_diff>
--- a/海外客诉台账_标准化数据.xlsx
+++ b/海外客诉台账_标准化数据.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="客诉明细" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据字典" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="客诉明细" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="数据字典" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
data: 自动同步石墨文档 2026-07-25 06:38
</commit_message>
<xml_diff>
--- a/海外客诉台账_标准化数据.xlsx
+++ b/海外客诉台账_标准化数据.xlsx
@@ -10767,7 +10767,7 @@
         <v>7</v>
       </c>
       <c r="AB73" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AC73" t="b">
         <v>0</v>
@@ -10782,7 +10782,7 @@
         <v>1</v>
       </c>
       <c r="AG73" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="74">

</xml_diff>